<commit_message>
Finalize AI agent workflow automation
</commit_message>
<xml_diff>
--- a/data/workflows/AI_Agent_Workflow_Assessment.xlsx
+++ b/data/workflows/AI_Agent_Workflow_Assessment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Questions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Workflows" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Test_Questions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -888,6 +888,48 @@
       <c r="H11" t="inlineStr">
         <is>
           <t>Performance summary with metrics, problem areas, and improvement recommendations</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WF011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Product Category Count</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>User asks how many products are in each category</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Product CSV</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Load products → Group products by category → Count products in each category → Generate category count report</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>If the product file contains no rows, return an appropriate empty-data result</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>CSV reader; aggregation/reporting</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Category names with product counts</t>
         </is>
       </c>
     </row>
@@ -902,7 +944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1092,6 +1134,23 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WF011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>How many products are in each category?</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Tests grouping, counting, and empty-data handling</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>